<commit_message>
New dataset generation merged npsy, erp and psd
</commit_message>
<xml_diff>
--- a/python/CaseStudy_1/outputs/results/CaseStudy_1_results.xlsx
+++ b/python/CaseStudy_1/outputs/results/CaseStudy_1_results.xlsx
@@ -552,12 +552,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>22.05 ± 2.92</t>
+          <t>21.63 ± 6.10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[16.72, 28.41]</t>
+          <t>[8.17, 30.00]</t>
         </is>
       </c>
     </row>
@@ -632,12 +632,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>375.27 ± 18.06</t>
+          <t>350.27 ± 18.06</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[338.60, 423.10]</t>
+          <t>[313.60, 398.10]</t>
         </is>
       </c>
     </row>
@@ -778,13 +778,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.3692164831711353</v>
+        <v>-0.2834915929037181</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01904745553823689</v>
+        <v>0.07628317966422776</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2446688430409396</v>
+        <v>0.2355355144361428</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1281131137744123</v>
+        <v>0.1434414278887164</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -1093,13 +1093,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.3312006574636533</v>
+        <v>0.2185720769811642</v>
       </c>
       <c r="D21" t="n">
-        <v>0.03683398881187383</v>
+        <v>0.1754221319580761</v>
       </c>
       <c r="E21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1219,13 +1219,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.3579763974372897</v>
+        <v>0.193628521063276</v>
       </c>
       <c r="D27" t="n">
-        <v>0.02332971593389057</v>
+        <v>0.2312474467715116</v>
       </c>
       <c r="E27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1324,10 +1324,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.2464844035752886</v>
+        <v>0.2784684926214037</v>
       </c>
       <c r="D32" t="n">
-        <v>0.125217577760777</v>
+        <v>0.0818689175462257</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1429,10 +1429,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.05882477596186395</v>
+        <v>0.1227150199789093</v>
       </c>
       <c r="D37" t="n">
-        <v>0.7184316571969948</v>
+        <v>0.4506299369860684</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1450,13 +1450,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-0.3869604318193696</v>
+        <v>-0.01048902954241881</v>
       </c>
       <c r="D38" t="n">
-        <v>0.01363686828041518</v>
+        <v>0.948781874753659</v>
       </c>
       <c r="E38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1471,10 +1471,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.005376337380531516</v>
+        <v>-0.1737427103182844</v>
       </c>
       <c r="D39" t="n">
-        <v>0.9737344688451568</v>
+        <v>0.2836384645112817</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1492,10 +1492,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.2395310425823124</v>
+        <v>-0.1777987171943505</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1365776913907301</v>
+        <v>0.2723730586470292</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1815,19 +1815,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-36.90762210701726</v>
+        <v>-38.05653659014764</v>
       </c>
       <c r="D6" t="n">
-        <v>48.08417925552223</v>
+        <v>47.02894543312258</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4427470338785884</v>
+        <v>0.4183913842490631</v>
       </c>
       <c r="F6" t="n">
-        <v>-131.1508816740088</v>
+        <v>-130.2315758699673</v>
       </c>
       <c r="G6" t="n">
-        <v>57.33563745997429</v>
+        <v>54.11850268967207</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1845,19 +1845,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.04595657932520025</v>
+        <v>-0.04595657932520032</v>
       </c>
       <c r="D7" t="n">
-        <v>0.07300693936642839</v>
+        <v>0.07300693936642831</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5290333241045782</v>
+        <v>0.5290333241045773</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1890475511048994</v>
+        <v>-0.1890475511048993</v>
       </c>
       <c r="G7" t="n">
-        <v>0.09713439245449887</v>
+        <v>0.09713439245449863</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -1875,19 +1875,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.833713566546275</v>
+        <v>3.83371356654628</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6439711402781579</v>
+        <v>0.6439711402781584</v>
       </c>
       <c r="E8" t="n">
-        <v>2.628883032767699e-09</v>
+        <v>2.628883032767623e-09</v>
       </c>
       <c r="F8" t="n">
-        <v>2.571553324517894</v>
+        <v>2.571553324517899</v>
       </c>
       <c r="G8" t="n">
-        <v>5.095873808574655</v>
+        <v>5.095873808574662</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
@@ -1905,19 +1905,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.07046515156812738</v>
+        <v>0.07046515156812835</v>
       </c>
       <c r="D9" t="n">
-        <v>0.07382882680094056</v>
+        <v>0.07382882680094055</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3398611991166866</v>
+        <v>0.33986119911668</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.07423668998256161</v>
+        <v>-0.07423668998256061</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2151669931188164</v>
+        <v>0.2151669931188173</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -1935,19 +1935,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.6782951320683159</v>
+        <v>-0.678295132068311</v>
       </c>
       <c r="D10" t="n">
         <v>1.227757567238736</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5806286652700792</v>
+        <v>0.5806286652700818</v>
       </c>
       <c r="F10" t="n">
-        <v>-3.084655745602753</v>
+        <v>-3.084655745602748</v>
       </c>
       <c r="G10" t="n">
-        <v>1.728065481466121</v>
+        <v>1.728065481466126</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1965,19 +1965,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.6580998767285238</v>
+        <v>-0.6580998767285248</v>
       </c>
       <c r="D11" t="n">
-        <v>0.146921634608142</v>
+        <v>0.1469216346081419</v>
       </c>
       <c r="E11" t="n">
-        <v>7.490302853563018e-06</v>
+        <v>7.490302853562755e-06</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.9460609891102356</v>
+        <v>-0.9460609891102365</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.3701387643468119</v>
+        <v>-0.370138764346813</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
@@ -1995,19 +1995,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.6761344601800641</v>
+        <v>-0.6761344601800605</v>
       </c>
       <c r="D12" t="n">
         <v>2.26044859478304</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7648521737475413</v>
+        <v>0.7648521737475424</v>
       </c>
       <c r="F12" t="n">
-        <v>-5.106532294858998</v>
+        <v>-5.106532294858995</v>
       </c>
       <c r="G12" t="n">
-        <v>3.75426337449887</v>
+        <v>3.754263374498874</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -2025,19 +2025,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.6194921040478576</v>
+        <v>0.6194921040478574</v>
       </c>
       <c r="D13" t="n">
         <v>0.1060352714646493</v>
       </c>
       <c r="E13" t="n">
-        <v>5.147845702556573e-09</v>
+        <v>5.147845702556687e-09</v>
       </c>
       <c r="F13" t="n">
-        <v>0.4116667908862172</v>
+        <v>0.4116667908862169</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8273174172094979</v>
+        <v>0.8273174172094978</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>

</xml_diff>